<commit_message>
Update: Status of 24.5.2026
</commit_message>
<xml_diff>
--- a/Einkommenssteuerberechnungen.xlsx
+++ b/Einkommenssteuerberechnungen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/preissl/Documents/Private/Finance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4029A8-A4D6-B941-922F-DE484F3F5546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EF588E-B545-2E42-8D27-3A24369A4488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26960" firstSheet="8" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2972,7 +2972,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17"/>
     <xf numFmtId="0" fontId="32" fillId="15" borderId="73"/>
   </cellStyleXfs>
-  <cellXfs count="348">
+  <cellXfs count="347">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3303,7 +3303,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="91" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="91" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="34" fillId="0" borderId="91" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -3423,23 +3422,6 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3448,6 +3430,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="10" borderId="80" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3461,6 +3449,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="84" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="85" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -4646,11 +4645,11 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="13" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="299" t="s">
+      <c r="B3" s="298" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="300"/>
-      <c r="D3" s="300"/>
+      <c r="C3" s="299"/>
+      <c r="D3" s="299"/>
     </row>
     <row r="7" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
@@ -4886,46 +4885,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="322"/>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="A1" s="321"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="320" t="s">
+      <c r="G1" s="319" t="s">
         <v>239</v>
       </c>
-      <c r="H1" s="306"/>
-      <c r="I1" s="306"/>
-      <c r="J1" s="306"/>
-      <c r="K1" s="306"/>
+      <c r="H1" s="305"/>
+      <c r="I1" s="305"/>
+      <c r="J1" s="305"/>
+      <c r="K1" s="305"/>
       <c r="L1" s="118"/>
-      <c r="M1" s="321" t="s">
+      <c r="M1" s="320" t="s">
         <v>240</v>
       </c>
-      <c r="N1" s="306"/>
-      <c r="O1" s="306"/>
-      <c r="P1" s="306"/>
-      <c r="Q1" s="292"/>
+      <c r="N1" s="305"/>
+      <c r="O1" s="305"/>
+      <c r="P1" s="305"/>
+      <c r="Q1" s="291"/>
     </row>
     <row r="2" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="317"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="316"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="300"/>
-      <c r="H2" s="300"/>
-      <c r="I2" s="300"/>
-      <c r="J2" s="300"/>
-      <c r="K2" s="300"/>
+      <c r="G2" s="299"/>
+      <c r="H2" s="299"/>
+      <c r="I2" s="299"/>
+      <c r="J2" s="299"/>
+      <c r="K2" s="299"/>
       <c r="L2" s="118"/>
-      <c r="M2" s="300"/>
-      <c r="N2" s="300"/>
-      <c r="O2" s="300"/>
-      <c r="P2" s="300"/>
-      <c r="Q2" s="303"/>
+      <c r="M2" s="299"/>
+      <c r="N2" s="299"/>
+      <c r="O2" s="299"/>
+      <c r="P2" s="299"/>
+      <c r="Q2" s="302"/>
     </row>
     <row r="3" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -5375,15 +5374,15 @@
       <c r="H15" s="59">
         <v>12.87</v>
       </c>
-      <c r="I15" s="294"/>
-      <c r="J15" s="314"/>
-      <c r="K15" s="296"/>
+      <c r="I15" s="293"/>
+      <c r="J15" s="313"/>
+      <c r="K15" s="295"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="O15" s="318"/>
-      <c r="P15" s="314"/>
-      <c r="Q15" s="296"/>
+      <c r="O15" s="317"/>
+      <c r="P15" s="313"/>
+      <c r="Q15" s="295"/>
     </row>
     <row r="16" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="144"/>
@@ -5505,13 +5504,13 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="323" t="s">
+      <c r="A21" s="322" t="s">
         <v>243</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -5526,11 +5525,11 @@
       <c r="Q21" s="10"/>
     </row>
     <row r="22" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -5779,10 +5778,10 @@
         <f>ROUND((B32-31000)*0.42+5950,2)</f>
         <v>9144.59</v>
       </c>
-      <c r="C33" s="301" t="s">
+      <c r="C33" s="300" t="s">
         <v>206</v>
       </c>
-      <c r="D33" s="296"/>
+      <c r="D33" s="295"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -5805,10 +5804,10 @@
         <f>ROUND((B13+H13+N13-620)*0.06,2)</f>
         <v>331.57</v>
       </c>
-      <c r="C34" s="301" t="s">
+      <c r="C34" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="296"/>
+      <c r="D34" s="295"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -6105,10 +6104,10 @@
       <c r="Q47" s="10"/>
     </row>
     <row r="48" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="304" t="s">
+      <c r="A48" s="303" t="s">
         <v>246</v>
       </c>
-      <c r="B48" s="292"/>
+      <c r="B48" s="291"/>
       <c r="C48" s="10"/>
       <c r="D48" s="10"/>
       <c r="E48" s="10"/>
@@ -8328,34 +8327,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="320" t="s">
+      <c r="A1" s="319" t="s">
         <v>257</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="321" t="s">
+      <c r="G1" s="320" t="s">
         <v>258</v>
       </c>
-      <c r="H1" s="306"/>
-      <c r="I1" s="306"/>
-      <c r="J1" s="306"/>
-      <c r="K1" s="292"/>
+      <c r="H1" s="305"/>
+      <c r="I1" s="305"/>
+      <c r="J1" s="305"/>
+      <c r="K1" s="291"/>
     </row>
     <row r="2" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="300"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="299"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="300"/>
-      <c r="H2" s="300"/>
-      <c r="I2" s="300"/>
-      <c r="J2" s="300"/>
-      <c r="K2" s="303"/>
+      <c r="G2" s="299"/>
+      <c r="H2" s="299"/>
+      <c r="I2" s="299"/>
+      <c r="J2" s="299"/>
+      <c r="K2" s="302"/>
     </row>
     <row r="3" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -8660,9 +8659,9 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="318"/>
-      <c r="J15" s="314"/>
-      <c r="K15" s="296"/>
+      <c r="I15" s="317"/>
+      <c r="J15" s="313"/>
+      <c r="K15" s="295"/>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="123" t="s">
@@ -8766,13 +8765,13 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="323" t="s">
+      <c r="A21" s="322" t="s">
         <v>259</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -8787,11 +8786,11 @@
       <c r="Q21" s="10"/>
     </row>
     <row r="22" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -9040,10 +9039,10 @@
         <f>ROUND((B32-31000)*0.42+5950,2)</f>
         <v>10076.74</v>
       </c>
-      <c r="C33" s="301" t="s">
+      <c r="C33" s="300" t="s">
         <v>206</v>
       </c>
-      <c r="D33" s="296"/>
+      <c r="D33" s="295"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -9066,10 +9065,10 @@
         <f>ROUND((B13+H13-620)*0.06,2)</f>
         <v>337.3</v>
       </c>
-      <c r="C34" s="301" t="s">
+      <c r="C34" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="296"/>
+      <c r="D34" s="295"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -9366,10 +9365,10 @@
       <c r="Q47" s="10"/>
     </row>
     <row r="48" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="304" t="s">
+      <c r="A48" s="303" t="s">
         <v>263</v>
       </c>
-      <c r="B48" s="292"/>
+      <c r="B48" s="291"/>
       <c r="C48" s="10"/>
       <c r="D48" s="10"/>
       <c r="E48" s="10"/>
@@ -11338,62 +11337,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="320" t="s">
+      <c r="A1" s="319" t="s">
         <v>273</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="321" t="s">
+      <c r="G1" s="320" t="s">
         <v>274</v>
       </c>
-      <c r="H1" s="306"/>
-      <c r="I1" s="306"/>
-      <c r="J1" s="306"/>
-      <c r="K1" s="292"/>
+      <c r="H1" s="305"/>
+      <c r="I1" s="305"/>
+      <c r="J1" s="305"/>
+      <c r="K1" s="291"/>
       <c r="L1" s="118"/>
-      <c r="M1" s="321" t="s">
+      <c r="M1" s="320" t="s">
         <v>275</v>
       </c>
-      <c r="N1" s="306"/>
-      <c r="O1" s="306"/>
-      <c r="P1" s="306"/>
-      <c r="Q1" s="292"/>
+      <c r="N1" s="305"/>
+      <c r="O1" s="305"/>
+      <c r="P1" s="305"/>
+      <c r="Q1" s="291"/>
       <c r="R1" s="118"/>
-      <c r="S1" s="321" t="s">
+      <c r="S1" s="320" t="s">
         <v>276</v>
       </c>
-      <c r="T1" s="306"/>
-      <c r="U1" s="306"/>
-      <c r="V1" s="306"/>
-      <c r="W1" s="292"/>
+      <c r="T1" s="305"/>
+      <c r="U1" s="305"/>
+      <c r="V1" s="305"/>
+      <c r="W1" s="291"/>
     </row>
     <row r="2" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="300"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="299"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="300"/>
-      <c r="H2" s="300"/>
-      <c r="I2" s="300"/>
-      <c r="J2" s="300"/>
-      <c r="K2" s="303"/>
+      <c r="G2" s="299"/>
+      <c r="H2" s="299"/>
+      <c r="I2" s="299"/>
+      <c r="J2" s="299"/>
+      <c r="K2" s="302"/>
       <c r="L2" s="118"/>
-      <c r="M2" s="300"/>
-      <c r="N2" s="300"/>
-      <c r="O2" s="300"/>
-      <c r="P2" s="300"/>
-      <c r="Q2" s="303"/>
+      <c r="M2" s="299"/>
+      <c r="N2" s="299"/>
+      <c r="O2" s="299"/>
+      <c r="P2" s="299"/>
+      <c r="Q2" s="302"/>
       <c r="R2" s="118"/>
-      <c r="S2" s="300"/>
-      <c r="T2" s="300"/>
-      <c r="U2" s="300"/>
-      <c r="V2" s="300"/>
-      <c r="W2" s="303"/>
+      <c r="S2" s="299"/>
+      <c r="T2" s="299"/>
+      <c r="U2" s="299"/>
+      <c r="V2" s="299"/>
+      <c r="W2" s="302"/>
     </row>
     <row r="3" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -11914,9 +11913,9 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="318"/>
-      <c r="J15" s="314"/>
-      <c r="K15" s="296"/>
+      <c r="I15" s="317"/>
+      <c r="J15" s="313"/>
+      <c r="K15" s="295"/>
       <c r="L15" s="10"/>
       <c r="M15" s="240" t="s">
         <v>11</v>
@@ -12096,13 +12095,13 @@
       <c r="W20" s="10"/>
     </row>
     <row r="21" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="323" t="s">
+      <c r="A21" s="322" t="s">
         <v>281</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -12122,11 +12121,11 @@
       <c r="W21" s="10"/>
     </row>
     <row r="22" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -12326,10 +12325,10 @@
         <f>ROUND((B30-60000)*0.48+1400+4225+12180,2)</f>
         <v>27569.02</v>
       </c>
-      <c r="C31" s="324" t="s">
+      <c r="C31" s="323" t="s">
         <v>283</v>
       </c>
-      <c r="D31" s="296"/>
+      <c r="D31" s="295"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
@@ -12352,10 +12351,10 @@
         <f>ROUND((B13+H13+N13-620)*0.06,2)</f>
         <v>420.11</v>
       </c>
-      <c r="C32" s="301" t="s">
+      <c r="C32" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="296"/>
+      <c r="D32" s="295"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
@@ -12581,12 +12580,12 @@
         <v>285</v>
       </c>
       <c r="D42" s="10"/>
-      <c r="E42" s="325" t="s">
+      <c r="E42" s="324" t="s">
         <v>286</v>
       </c>
-      <c r="F42" s="314"/>
-      <c r="G42" s="314"/>
-      <c r="H42" s="296"/>
+      <c r="F42" s="313"/>
+      <c r="G42" s="313"/>
+      <c r="H42" s="295"/>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
       <c r="K42" s="10"/>
@@ -12677,10 +12676,10 @@
       <c r="Q45" s="10"/>
     </row>
     <row r="46" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="304" t="s">
+      <c r="A46" s="303" t="s">
         <v>290</v>
       </c>
-      <c r="B46" s="292"/>
+      <c r="B46" s="291"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="248" t="s">
@@ -13953,21 +13952,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="320" t="s">
+      <c r="A1" s="319" t="s">
         <v>298</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
     </row>
     <row r="2" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="300"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="299"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
     </row>
     <row r="3" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14183,21 +14182,21 @@
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="323" t="s">
+      <c r="A21" s="322" t="s">
         <v>299</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
     </row>
     <row r="22" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
     </row>
     <row r="23" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14298,10 +14297,10 @@
         <f>ROUND((B30-93120)*0.5+32571.75,2)</f>
         <v>34026.410000000003</v>
       </c>
-      <c r="C31" s="324" t="s">
+      <c r="C31" s="323" t="s">
         <v>23</v>
       </c>
-      <c r="D31" s="296"/>
+      <c r="D31" s="295"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
     </row>
@@ -14313,10 +14312,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>894.01</v>
       </c>
-      <c r="C32" s="301" t="s">
+      <c r="C32" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="296"/>
+      <c r="D32" s="295"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
     </row>
@@ -14428,22 +14427,22 @@
         <f>B39-B40</f>
         <v>-924.99999999999625</v>
       </c>
-      <c r="C42" s="293" t="s">
+      <c r="C42" s="292" t="s">
         <v>301</v>
       </c>
-      <c r="D42" s="296"/>
-      <c r="E42" s="326" t="s">
+      <c r="D42" s="295"/>
+      <c r="E42" s="325" t="s">
         <v>33</v>
       </c>
-      <c r="F42" s="314"/>
+      <c r="F42" s="313"/>
     </row>
     <row r="43" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="57"/>
       <c r="B43" s="57"/>
-      <c r="C43" s="327" t="s">
+      <c r="C43" s="326" t="s">
         <v>302</v>
       </c>
-      <c r="D43" s="296"/>
+      <c r="D43" s="295"/>
       <c r="E43" s="248" t="s">
         <v>35</v>
       </c>
@@ -14479,10 +14478,10 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="304" t="s">
+      <c r="A46" s="303" t="s">
         <v>38</v>
       </c>
-      <c r="B46" s="292"/>
+      <c r="B46" s="291"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="248" t="s">
@@ -15733,21 +15732,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="320" t="s">
+      <c r="A1" s="319" t="s">
         <v>312</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
     </row>
     <row r="2" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="300"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="299"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
     </row>
     <row r="3" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -15963,21 +15962,21 @@
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="323" t="s">
+      <c r="A21" s="322" t="s">
         <v>313</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
     </row>
     <row r="22" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
     </row>
     <row r="23" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -16118,10 +16117,10 @@
         <f>ROUND((B33-99266)*0.5+34222.42,2)</f>
         <v>44541.03</v>
       </c>
-      <c r="C34" s="324" t="s">
+      <c r="C34" s="323" t="s">
         <v>23</v>
       </c>
-      <c r="D34" s="296"/>
+      <c r="D34" s="295"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
     </row>
@@ -16133,10 +16132,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>1186.67</v>
       </c>
-      <c r="C35" s="301" t="s">
+      <c r="C35" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="296"/>
+      <c r="D35" s="295"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
     </row>
@@ -16248,14 +16247,14 @@
         <f>B42-B43</f>
         <v>-646.00000000000227</v>
       </c>
-      <c r="C45" s="293" t="s">
+      <c r="C45" s="292" t="s">
         <v>316</v>
       </c>
-      <c r="D45" s="296"/>
-      <c r="E45" s="326" t="s">
+      <c r="D45" s="295"/>
+      <c r="E45" s="325" t="s">
         <v>33</v>
       </c>
-      <c r="F45" s="314"/>
+      <c r="F45" s="313"/>
     </row>
     <row r="46" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="57"/>
@@ -16299,10 +16298,10 @@
       </c>
     </row>
     <row r="49" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="304" t="s">
+      <c r="A49" s="303" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="292"/>
+      <c r="B49" s="291"/>
       <c r="C49" s="10"/>
       <c r="D49" s="10"/>
       <c r="E49" s="248" t="s">
@@ -18543,23 +18542,23 @@
     <col min="1" max="1" width="53.25" customWidth="1"/>
     <col min="2" max="2" width="16.5" customWidth="1"/>
     <col min="3" max="3" width="16.625" customWidth="1"/>
-    <col min="4" max="4" width="39.625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="21.125" customWidth="1"/>
     <col min="6" max="6" width="12.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="290" t="s">
+      <c r="A1" s="289" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="290"/>
-      <c r="C1" s="290"/>
+      <c r="B1" s="289"/>
+      <c r="C1" s="289"/>
       <c r="D1" s="272"/>
     </row>
     <row r="2" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="290"/>
-      <c r="B2" s="290"/>
-      <c r="C2" s="290"/>
+      <c r="A2" s="289"/>
+      <c r="B2" s="289"/>
+      <c r="C2" s="289"/>
     </row>
     <row r="3" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -18706,23 +18705,23 @@
       <c r="B17" s="62">
         <v>53694.19</v>
       </c>
-      <c r="C17" s="285">
+      <c r="C17" s="284">
         <v>260</v>
       </c>
       <c r="D17" s="10"/>
     </row>
     <row r="18" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="290" t="s">
+      <c r="A18" s="289" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="290"/>
-      <c r="C18" s="290"/>
+      <c r="B18" s="289"/>
+      <c r="C18" s="289"/>
       <c r="D18" s="273"/>
     </row>
     <row r="19" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="290"/>
-      <c r="B19" s="290"/>
-      <c r="C19" s="290"/>
+      <c r="A19" s="289"/>
+      <c r="B19" s="289"/>
+      <c r="C19" s="289"/>
       <c r="D19" s="274"/>
     </row>
     <row r="20" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -18834,10 +18833,10 @@
         <f>ROUND((B29-103072)*0.5+35534.38,2)</f>
         <v>52245.8</v>
       </c>
-      <c r="C30" s="293" t="s">
+      <c r="C30" s="292" t="s">
         <v>23</v>
       </c>
-      <c r="D30" s="294"/>
+      <c r="D30" s="293"/>
     </row>
     <row r="31" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="52" t="s">
@@ -18847,10 +18846,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>1301.33</v>
       </c>
-      <c r="C31" s="295" t="s">
+      <c r="C31" s="294" t="s">
         <v>25</v>
       </c>
-      <c r="D31" s="294"/>
+      <c r="D31" s="293"/>
     </row>
     <row r="32" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="82" t="s">
@@ -18932,10 +18931,10 @@
         <f>B38</f>
         <v>-649.99999999999773</v>
       </c>
-      <c r="C40" s="293" t="s">
+      <c r="C40" s="292" t="s">
         <v>32</v>
       </c>
-      <c r="D40" s="296"/>
+      <c r="D40" s="295"/>
     </row>
     <row r="41" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="57"/>
@@ -18958,10 +18957,10 @@
       <c r="D43" s="10"/>
     </row>
     <row r="44" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="291" t="s">
+      <c r="A44" s="290" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="292"/>
+      <c r="B44" s="291"/>
       <c r="C44" s="10"/>
       <c r="D44" s="10"/>
     </row>
@@ -19024,10 +19023,10 @@
       <c r="D50" s="119"/>
     </row>
     <row r="51" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="284" t="s">
+      <c r="A51" s="283" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="283">
+      <c r="B51" s="282">
         <f>B45-B46-B47+B48</f>
         <v>108496.34000000001</v>
       </c>
@@ -19036,12 +19035,12 @@
     </row>
     <row r="52" spans="1:4" ht="19" x14ac:dyDescent="0.2"/>
     <row r="54" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="297" t="s">
+      <c r="A54" s="296" t="s">
         <v>459</v>
       </c>
-      <c r="B54" s="298"/>
-      <c r="C54" s="298"/>
-      <c r="D54" s="298"/>
+      <c r="B54" s="297"/>
+      <c r="C54" s="297"/>
+      <c r="D54" s="297"/>
     </row>
     <row r="55" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="248" t="s">
@@ -19071,94 +19070,94 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="286" t="s">
+      <c r="A59" s="285" t="s">
         <v>460</v>
       </c>
-      <c r="B59" s="287"/>
-      <c r="C59" s="287"/>
-      <c r="D59" s="287"/>
+      <c r="B59" s="286"/>
+      <c r="C59" s="286"/>
+      <c r="D59" s="286"/>
     </row>
     <row r="60" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="281" t="s">
+      <c r="A60" s="280" t="s">
         <v>39</v>
       </c>
-      <c r="B60" s="276">
+      <c r="B60" s="279">
         <v>6773</v>
       </c>
       <c r="C60" s="275" t="s">
         <v>40</v>
       </c>
-      <c r="D60" s="280">
+      <c r="D60" s="279">
         <v>7518.44</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="281" t="s">
+      <c r="A61" s="280" t="s">
         <v>42</v>
       </c>
-      <c r="B61" s="276">
+      <c r="B61" s="279">
         <v>7341.69</v>
       </c>
       <c r="C61" s="275" t="s">
         <v>43</v>
       </c>
-      <c r="D61" s="280">
+      <c r="D61" s="279">
         <v>6637.88</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="281" t="s">
+      <c r="A62" s="280" t="s">
         <v>45</v>
       </c>
-      <c r="B62" s="276">
+      <c r="B62" s="279">
         <v>7121.67</v>
       </c>
       <c r="C62" s="275" t="s">
         <v>46</v>
       </c>
-      <c r="D62" s="280">
+      <c r="D62" s="279">
         <v>6888.36</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="281" t="s">
+      <c r="A63" s="280" t="s">
         <v>47</v>
       </c>
-      <c r="B63" s="276">
+      <c r="B63" s="279">
         <v>7138.6</v>
       </c>
       <c r="C63" s="275" t="s">
         <v>48</v>
       </c>
-      <c r="D63" s="280">
+      <c r="D63" s="279">
         <v>17811.8</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="281" t="s">
+      <c r="A64" s="280" t="s">
         <v>50</v>
       </c>
-      <c r="B64" s="276">
+      <c r="B64" s="279">
         <v>6773.36</v>
       </c>
       <c r="C64" s="275" t="s">
         <v>51</v>
       </c>
-      <c r="D64" s="280">
+      <c r="D64" s="279">
         <v>15441.21</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="281" t="s">
+      <c r="A65" s="280" t="s">
         <v>53</v>
       </c>
-      <c r="B65" s="276">
+      <c r="B65" s="279">
         <v>13789.38</v>
       </c>
       <c r="C65" s="275" t="s">
         <v>54</v>
       </c>
-      <c r="D65" s="280">
+      <c r="D65" s="279">
         <v>7717.5</v>
       </c>
     </row>
@@ -19166,64 +19165,64 @@
       <c r="A66" s="249"/>
     </row>
     <row r="67" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="288" t="s">
+      <c r="A67" s="287" t="s">
         <v>453</v>
       </c>
-      <c r="B67" s="289"/>
-      <c r="C67" s="289"/>
+      <c r="B67" s="288"/>
+      <c r="C67" s="288"/>
     </row>
     <row r="68" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="282" t="s">
+      <c r="A68" s="281" t="s">
         <v>454</v>
       </c>
-      <c r="B68" s="277">
+      <c r="B68" s="276">
         <v>19337.919999999998</v>
       </c>
-      <c r="C68" s="277">
+      <c r="C68" s="276">
         <v>27198.92</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="282" t="s">
+      <c r="A69" s="281" t="s">
         <v>455</v>
       </c>
-      <c r="B69" s="278">
+      <c r="B69" s="277">
         <v>5294.12</v>
       </c>
-      <c r="C69" s="279">
+      <c r="C69" s="278">
         <v>6534.84</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="282" t="s">
+      <c r="A70" s="281" t="s">
         <v>456</v>
       </c>
-      <c r="B70" s="279">
+      <c r="B70" s="278">
         <v>7497.68</v>
       </c>
-      <c r="C70" s="279">
+      <c r="C70" s="278">
         <v>9012.9599999999991</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="282" t="s">
+      <c r="A71" s="281" t="s">
         <v>457</v>
       </c>
-      <c r="B71" s="277">
+      <c r="B71" s="276">
         <v>0</v>
       </c>
-      <c r="C71" s="277">
+      <c r="C71" s="276">
         <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="282" t="s">
+      <c r="A72" s="281" t="s">
         <v>457</v>
       </c>
-      <c r="B72" s="277">
+      <c r="B72" s="276">
         <v>0</v>
       </c>
-      <c r="C72" s="277">
+      <c r="C72" s="276">
         <v>0</v>
       </c>
     </row>
@@ -19708,11 +19707,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="341" t="s">
+      <c r="A1" s="335" t="s">
         <v>327</v>
       </c>
-      <c r="B1" s="342"/>
-      <c r="C1" s="343"/>
+      <c r="B1" s="336"/>
+      <c r="C1" s="337"/>
       <c r="D1" s="159"/>
       <c r="E1" s="39" t="s">
         <v>328</v>
@@ -19880,11 +19879,11 @@
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="338" t="s">
+      <c r="A11" s="328" t="s">
         <v>344</v>
       </c>
-      <c r="B11" s="339"/>
-      <c r="C11" s="340"/>
+      <c r="B11" s="329"/>
+      <c r="C11" s="330"/>
       <c r="D11" s="159"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -20068,11 +20067,11 @@
       <c r="J22" s="10"/>
     </row>
     <row r="23" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="338" t="s">
+      <c r="A23" s="328" t="s">
         <v>355</v>
       </c>
-      <c r="B23" s="339"/>
-      <c r="C23" s="340"/>
+      <c r="B23" s="329"/>
+      <c r="C23" s="330"/>
       <c r="D23" s="159"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -20348,11 +20347,11 @@
       <c r="J39" s="10"/>
     </row>
     <row r="40" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="345" t="s">
+      <c r="A40" s="339" t="s">
         <v>371</v>
       </c>
-      <c r="B40" s="346"/>
-      <c r="C40" s="347"/>
+      <c r="B40" s="340"/>
+      <c r="C40" s="341"/>
       <c r="D40" s="159"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -20444,13 +20443,13 @@
       <c r="C46" s="212">
         <v>-604</v>
       </c>
-      <c r="D46" s="337"/>
-      <c r="E46" s="314"/>
-      <c r="F46" s="314"/>
-      <c r="G46" s="314"/>
-      <c r="H46" s="314"/>
-      <c r="I46" s="314"/>
-      <c r="J46" s="296"/>
+      <c r="D46" s="327"/>
+      <c r="E46" s="313"/>
+      <c r="F46" s="313"/>
+      <c r="G46" s="313"/>
+      <c r="H46" s="313"/>
+      <c r="I46" s="313"/>
+      <c r="J46" s="295"/>
     </row>
     <row r="47" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="175" t="s">
@@ -20584,11 +20583,11 @@
       <c r="J54" s="10"/>
     </row>
     <row r="55" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="332" t="s">
+      <c r="A55" s="342" t="s">
         <v>383</v>
       </c>
-      <c r="B55" s="333"/>
-      <c r="C55" s="334"/>
+      <c r="B55" s="343"/>
+      <c r="C55" s="344"/>
       <c r="D55" s="215"/>
       <c r="E55" s="10"/>
       <c r="F55" s="10"/>
@@ -20899,10 +20898,10 @@
       <c r="J75" s="10"/>
     </row>
     <row r="76" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="344" t="s">
+      <c r="A76" s="338" t="s">
         <v>399</v>
       </c>
-      <c r="B76" s="300"/>
+      <c r="B76" s="299"/>
       <c r="C76" s="60"/>
       <c r="D76" s="10"/>
       <c r="E76" s="10"/>
@@ -20913,8 +20912,8 @@
       <c r="J76" s="10"/>
     </row>
     <row r="77" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="317"/>
-      <c r="B77" s="300"/>
+      <c r="A77" s="316"/>
+      <c r="B77" s="299"/>
       <c r="C77" s="60"/>
       <c r="D77" s="10"/>
       <c r="E77" s="10"/>
@@ -20953,10 +20952,10 @@
       <c r="J79" s="10"/>
     </row>
     <row r="80" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="335" t="s">
+      <c r="A80" s="345" t="s">
         <v>402</v>
       </c>
-      <c r="B80" s="308"/>
+      <c r="B80" s="307"/>
       <c r="C80" s="60"/>
       <c r="D80" s="10"/>
       <c r="E80" s="10"/>
@@ -20967,8 +20966,8 @@
       <c r="J80" s="10"/>
     </row>
     <row r="81" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="317"/>
-      <c r="B81" s="300"/>
+      <c r="A81" s="316"/>
+      <c r="B81" s="299"/>
       <c r="C81" s="60"/>
       <c r="D81" s="10"/>
       <c r="E81" s="10"/>
@@ -21175,10 +21174,10 @@
       <c r="J95" s="10"/>
     </row>
     <row r="96" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="328" t="s">
+      <c r="A96" s="331" t="s">
         <v>417</v>
       </c>
-      <c r="B96" s="329"/>
+      <c r="B96" s="332"/>
       <c r="C96" s="10"/>
       <c r="D96" s="10"/>
       <c r="E96" s="10"/>
@@ -21189,8 +21188,8 @@
       <c r="J96" s="10"/>
     </row>
     <row r="97" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="330"/>
-      <c r="B97" s="331"/>
+      <c r="A97" s="333"/>
+      <c r="B97" s="334"/>
       <c r="C97" s="10"/>
       <c r="D97" s="10"/>
       <c r="E97" s="10"/>
@@ -21339,14 +21338,14 @@
       <c r="B108" s="10"/>
     </row>
     <row r="109" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="336" t="s">
+      <c r="A109" s="346" t="s">
         <v>429</v>
       </c>
-      <c r="B109" s="329"/>
+      <c r="B109" s="332"/>
     </row>
     <row r="110" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="330"/>
-      <c r="B110" s="331"/>
+      <c r="A110" s="333"/>
+      <c r="B110" s="334"/>
     </row>
     <row r="111" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="236" t="s">
@@ -21418,14 +21417,14 @@
       </c>
     </row>
     <row r="124" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="328" t="s">
+      <c r="A124" s="331" t="s">
         <v>443</v>
       </c>
-      <c r="B124" s="329"/>
+      <c r="B124" s="332"/>
     </row>
     <row r="125" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="330"/>
-      <c r="B125" s="331"/>
+      <c r="A125" s="333"/>
+      <c r="B125" s="334"/>
     </row>
     <row r="126" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="225" t="s">
@@ -21444,14 +21443,14 @@
       </c>
     </row>
     <row r="128" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="328" t="s">
+      <c r="A128" s="331" t="s">
         <v>448</v>
       </c>
-      <c r="B128" s="329"/>
+      <c r="B128" s="332"/>
     </row>
     <row r="129" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="330"/>
-      <c r="B129" s="331"/>
+      <c r="A129" s="333"/>
+      <c r="B129" s="334"/>
     </row>
     <row r="130" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="225" t="s">
@@ -21471,6 +21470,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A124:B125"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A80:B81"/>
+    <mergeCell ref="A128:B129"/>
+    <mergeCell ref="A109:B110"/>
     <mergeCell ref="D46:J46"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A96:B97"/>
@@ -21478,11 +21482,6 @@
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A76:B77"/>
     <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A124:B125"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A80:B81"/>
-    <mergeCell ref="A128:B129"/>
-    <mergeCell ref="A109:B110"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
@@ -22643,20 +22642,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="305" t="s">
+      <c r="A1" s="304" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="292"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="291"/>
     </row>
     <row r="2" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="302"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="303"/>
+      <c r="A2" s="301"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="302"/>
     </row>
     <row r="3" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -22816,11 +22815,11 @@
       <c r="B15" s="59">
         <v>438.04</v>
       </c>
-      <c r="C15" s="313" t="s">
+      <c r="C15" s="312" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="314"/>
-      <c r="E15" s="296"/>
+      <c r="D15" s="313"/>
+      <c r="E15" s="295"/>
     </row>
     <row r="16" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="58" t="s">
@@ -22868,20 +22867,20 @@
       <c r="E20" s="49"/>
     </row>
     <row r="21" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="307" t="s">
+      <c r="A21" s="306" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
     </row>
     <row r="22" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
     </row>
     <row r="23" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="63" t="s">
@@ -23009,10 +23008,10 @@
         <f>ROUND((B33-18000)*0.35+1750,2)</f>
         <v>5779.41</v>
       </c>
-      <c r="C34" s="301" t="s">
+      <c r="C34" s="300" t="s">
         <v>142</v>
       </c>
-      <c r="D34" s="296"/>
+      <c r="D34" s="295"/>
       <c r="E34" s="10"/>
     </row>
     <row r="35" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -23023,10 +23022,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>244.34</v>
       </c>
-      <c r="C35" s="301" t="s">
+      <c r="C35" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="296"/>
+      <c r="D35" s="295"/>
       <c r="E35" s="10"/>
     </row>
     <row r="36" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -23153,10 +23152,10 @@
       <c r="E48" s="10"/>
     </row>
     <row r="49" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="304" t="s">
+      <c r="A49" s="303" t="s">
         <v>147</v>
       </c>
-      <c r="B49" s="292"/>
+      <c r="B49" s="291"/>
       <c r="C49" s="10"/>
       <c r="D49" s="10"/>
       <c r="E49" s="10"/>
@@ -26527,34 +26526,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="316" t="s">
+      <c r="A1" s="315" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="315" t="s">
+      <c r="G1" s="314" t="s">
         <v>199</v>
       </c>
-      <c r="H1" s="306"/>
-      <c r="I1" s="306"/>
-      <c r="J1" s="306"/>
-      <c r="K1" s="292"/>
+      <c r="H1" s="305"/>
+      <c r="I1" s="305"/>
+      <c r="J1" s="305"/>
+      <c r="K1" s="291"/>
     </row>
     <row r="2" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="317"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="316"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="300"/>
-      <c r="H2" s="300"/>
-      <c r="I2" s="300"/>
-      <c r="J2" s="300"/>
-      <c r="K2" s="303"/>
+      <c r="G2" s="299"/>
+      <c r="H2" s="299"/>
+      <c r="I2" s="299"/>
+      <c r="J2" s="299"/>
+      <c r="K2" s="302"/>
     </row>
     <row r="3" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -26853,11 +26852,11 @@
       <c r="B15" s="59">
         <v>1535.69</v>
       </c>
-      <c r="C15" s="313" t="s">
+      <c r="C15" s="312" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="314"/>
-      <c r="E15" s="296"/>
+      <c r="D15" s="313"/>
+      <c r="E15" s="295"/>
       <c r="F15" s="119"/>
       <c r="G15" s="123" t="s">
         <v>132</v>
@@ -26865,11 +26864,11 @@
       <c r="H15" s="59">
         <v>413.13</v>
       </c>
-      <c r="I15" s="313" t="s">
+      <c r="I15" s="312" t="s">
         <v>133</v>
       </c>
-      <c r="J15" s="314"/>
-      <c r="K15" s="296"/>
+      <c r="J15" s="313"/>
+      <c r="K15" s="295"/>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="58" t="s">
@@ -26957,13 +26956,13 @@
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="307" t="s">
+      <c r="A21" s="306" t="s">
         <v>203</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -26972,11 +26971,11 @@
       <c r="K21" s="10"/>
     </row>
     <row r="22" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -27177,10 +27176,10 @@
         <f>ROUND((B33-31000)*0.42+6300,2)</f>
         <v>7196.73</v>
       </c>
-      <c r="C34" s="301" t="s">
+      <c r="C34" s="300" t="s">
         <v>206</v>
       </c>
-      <c r="D34" s="296"/>
+      <c r="D34" s="295"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -27197,10 +27196,10 @@
         <f>ROUND((B13+H13-620)*0.06,2)</f>
         <v>312.08999999999997</v>
       </c>
-      <c r="C35" s="301" t="s">
+      <c r="C35" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="296"/>
+      <c r="D35" s="295"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
@@ -27424,10 +27423,10 @@
       <c r="K49" s="10"/>
     </row>
     <row r="50" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="304" t="s">
+      <c r="A50" s="303" t="s">
         <v>208</v>
       </c>
-      <c r="B50" s="292"/>
+      <c r="B50" s="291"/>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
@@ -31189,48 +31188,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="316" t="s">
+      <c r="A1" s="315" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
+      <c r="B1" s="305"/>
+      <c r="C1" s="305"/>
+      <c r="D1" s="305"/>
+      <c r="E1" s="305"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="319" t="s">
+      <c r="G1" s="318" t="s">
         <v>222</v>
       </c>
-      <c r="H1" s="306"/>
-      <c r="I1" s="306"/>
-      <c r="J1" s="306"/>
-      <c r="K1" s="306"/>
+      <c r="H1" s="305"/>
+      <c r="I1" s="305"/>
+      <c r="J1" s="305"/>
+      <c r="K1" s="305"/>
       <c r="L1" s="118"/>
-      <c r="M1" s="315" t="s">
+      <c r="M1" s="314" t="s">
         <v>223</v>
       </c>
-      <c r="N1" s="306"/>
-      <c r="O1" s="306"/>
-      <c r="P1" s="306"/>
-      <c r="Q1" s="292"/>
+      <c r="N1" s="305"/>
+      <c r="O1" s="305"/>
+      <c r="P1" s="305"/>
+      <c r="Q1" s="291"/>
     </row>
     <row r="2" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="317"/>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="316"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="300"/>
-      <c r="H2" s="300"/>
-      <c r="I2" s="300"/>
-      <c r="J2" s="300"/>
-      <c r="K2" s="300"/>
+      <c r="G2" s="299"/>
+      <c r="H2" s="299"/>
+      <c r="I2" s="299"/>
+      <c r="J2" s="299"/>
+      <c r="K2" s="299"/>
       <c r="L2" s="118"/>
-      <c r="M2" s="300"/>
-      <c r="N2" s="300"/>
-      <c r="O2" s="300"/>
-      <c r="P2" s="300"/>
-      <c r="Q2" s="303"/>
+      <c r="M2" s="299"/>
+      <c r="N2" s="299"/>
+      <c r="O2" s="299"/>
+      <c r="P2" s="299"/>
+      <c r="Q2" s="302"/>
     </row>
     <row r="3" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -31668,11 +31667,11 @@
       <c r="B15" s="59">
         <v>175.89</v>
       </c>
-      <c r="C15" s="313" t="s">
+      <c r="C15" s="312" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="314"/>
-      <c r="E15" s="296"/>
+      <c r="D15" s="313"/>
+      <c r="E15" s="295"/>
       <c r="F15" s="119"/>
       <c r="G15" s="123" t="s">
         <v>132</v>
@@ -31680,17 +31679,17 @@
       <c r="H15" s="59">
         <v>13.93</v>
       </c>
-      <c r="I15" s="313" t="s">
+      <c r="I15" s="312" t="s">
         <v>133</v>
       </c>
-      <c r="J15" s="314"/>
-      <c r="K15" s="296"/>
+      <c r="J15" s="313"/>
+      <c r="K15" s="295"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="O15" s="318"/>
-      <c r="P15" s="314"/>
-      <c r="Q15" s="296"/>
+      <c r="O15" s="317"/>
+      <c r="P15" s="313"/>
+      <c r="Q15" s="295"/>
     </row>
     <row r="16" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="58" t="s">
@@ -31814,13 +31813,13 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="307" t="s">
+      <c r="A21" s="306" t="s">
         <v>227</v>
       </c>
-      <c r="B21" s="308"/>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="309"/>
+      <c r="B21" s="307"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="307"/>
+      <c r="E21" s="308"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -31835,11 +31834,11 @@
       <c r="Q21" s="10"/>
     </row>
     <row r="22" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="310"/>
-      <c r="B22" s="311"/>
-      <c r="C22" s="311"/>
-      <c r="D22" s="311"/>
-      <c r="E22" s="312"/>
+      <c r="A22" s="309"/>
+      <c r="B22" s="310"/>
+      <c r="C22" s="310"/>
+      <c r="D22" s="310"/>
+      <c r="E22" s="311"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -32088,10 +32087,10 @@
         <f>ROUND((B32-31000)*0.42+6300,2)</f>
         <v>8538.18</v>
       </c>
-      <c r="C33" s="301" t="s">
+      <c r="C33" s="300" t="s">
         <v>206</v>
       </c>
-      <c r="D33" s="296"/>
+      <c r="D33" s="295"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -32114,10 +32113,10 @@
         <f>ROUND((B13+H13+N13-620)*0.06,2)</f>
         <v>329.36</v>
       </c>
-      <c r="C34" s="301" t="s">
+      <c r="C34" s="300" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="296"/>
+      <c r="D34" s="295"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -32395,10 +32394,10 @@
       <c r="Q46" s="10"/>
     </row>
     <row r="47" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="304" t="s">
+      <c r="A47" s="303" t="s">
         <v>230</v>
       </c>
-      <c r="B47" s="292"/>
+      <c r="B47" s="291"/>
       <c r="C47" s="10"/>
       <c r="D47" s="10"/>
       <c r="E47" s="10"/>

</xml_diff>

<commit_message>
Update Costs for Immo in Corneliusgasse
</commit_message>
<xml_diff>
--- a/Einkommenssteuerberechnungen.xlsx
+++ b/Einkommenssteuerberechnungen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/preissl/Documents/Private/Finance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD4E528A-8716-F945-AE97-C22F8A0CA963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253ED2EC-1D0D-7445-9004-41A9D410A5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="1980" windowWidth="34560" windowHeight="21680" firstSheet="8" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20440" firstSheet="8" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -3337,9 +3337,6 @@
     <xf numFmtId="49" fontId="22" fillId="6" borderId="91" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="31" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3351,6 +3348,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="17" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -3416,23 +3419,6 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3441,6 +3427,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="10" borderId="80" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3454,12 +3446,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="84" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="85" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="17" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="29" fillId="10" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -4645,11 +4643,11 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="13" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="296" t="s">
+      <c r="B3" s="297" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="297"/>
-      <c r="D3" s="297"/>
+      <c r="C3" s="298"/>
+      <c r="D3" s="298"/>
     </row>
     <row r="7" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
@@ -4885,46 +4883,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="319"/>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="A1" s="320"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="317" t="s">
+      <c r="G1" s="318" t="s">
         <v>238</v>
       </c>
-      <c r="H1" s="303"/>
-      <c r="I1" s="303"/>
-      <c r="J1" s="303"/>
-      <c r="K1" s="303"/>
+      <c r="H1" s="304"/>
+      <c r="I1" s="304"/>
+      <c r="J1" s="304"/>
+      <c r="K1" s="304"/>
       <c r="L1" s="118"/>
-      <c r="M1" s="318" t="s">
+      <c r="M1" s="319" t="s">
         <v>239</v>
       </c>
-      <c r="N1" s="303"/>
-      <c r="O1" s="303"/>
-      <c r="P1" s="303"/>
-      <c r="Q1" s="291"/>
+      <c r="N1" s="304"/>
+      <c r="O1" s="304"/>
+      <c r="P1" s="304"/>
+      <c r="Q1" s="290"/>
     </row>
     <row r="2" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="314"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="315"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="297"/>
-      <c r="H2" s="297"/>
-      <c r="I2" s="297"/>
-      <c r="J2" s="297"/>
-      <c r="K2" s="297"/>
+      <c r="G2" s="298"/>
+      <c r="H2" s="298"/>
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="298"/>
       <c r="L2" s="118"/>
-      <c r="M2" s="297"/>
-      <c r="N2" s="297"/>
-      <c r="O2" s="297"/>
-      <c r="P2" s="297"/>
-      <c r="Q2" s="300"/>
+      <c r="M2" s="298"/>
+      <c r="N2" s="298"/>
+      <c r="O2" s="298"/>
+      <c r="P2" s="298"/>
+      <c r="Q2" s="301"/>
     </row>
     <row r="3" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -5374,15 +5372,15 @@
       <c r="H15" s="59">
         <v>12.87</v>
       </c>
-      <c r="I15" s="293"/>
-      <c r="J15" s="311"/>
-      <c r="K15" s="295"/>
+      <c r="I15" s="292"/>
+      <c r="J15" s="312"/>
+      <c r="K15" s="294"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="O15" s="315"/>
-      <c r="P15" s="311"/>
-      <c r="Q15" s="295"/>
+      <c r="O15" s="316"/>
+      <c r="P15" s="312"/>
+      <c r="Q15" s="294"/>
     </row>
     <row r="16" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="144"/>
@@ -5504,13 +5502,13 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="320" t="s">
+      <c r="A21" s="321" t="s">
         <v>242</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -5525,11 +5523,11 @@
       <c r="Q21" s="10"/>
     </row>
     <row r="22" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -5778,10 +5776,10 @@
         <f>ROUND((B32-31000)*0.42+5950,2)</f>
         <v>9144.59</v>
       </c>
-      <c r="C33" s="298" t="s">
+      <c r="C33" s="299" t="s">
         <v>205</v>
       </c>
-      <c r="D33" s="295"/>
+      <c r="D33" s="294"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -5804,10 +5802,10 @@
         <f>ROUND((B13+H13+N13-620)*0.06,2)</f>
         <v>331.57</v>
       </c>
-      <c r="C34" s="298" t="s">
+      <c r="C34" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="295"/>
+      <c r="D34" s="294"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -6104,10 +6102,10 @@
       <c r="Q47" s="10"/>
     </row>
     <row r="48" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="301" t="s">
+      <c r="A48" s="302" t="s">
         <v>245</v>
       </c>
-      <c r="B48" s="291"/>
+      <c r="B48" s="290"/>
       <c r="C48" s="10"/>
       <c r="D48" s="10"/>
       <c r="E48" s="10"/>
@@ -8327,34 +8325,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="317" t="s">
+      <c r="A1" s="318" t="s">
         <v>256</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="318" t="s">
+      <c r="G1" s="319" t="s">
         <v>257</v>
       </c>
-      <c r="H1" s="303"/>
-      <c r="I1" s="303"/>
-      <c r="J1" s="303"/>
-      <c r="K1" s="291"/>
+      <c r="H1" s="304"/>
+      <c r="I1" s="304"/>
+      <c r="J1" s="304"/>
+      <c r="K1" s="290"/>
     </row>
     <row r="2" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="297"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="298"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="297"/>
-      <c r="H2" s="297"/>
-      <c r="I2" s="297"/>
-      <c r="J2" s="297"/>
-      <c r="K2" s="300"/>
+      <c r="G2" s="298"/>
+      <c r="H2" s="298"/>
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="301"/>
     </row>
     <row r="3" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -8659,9 +8657,9 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="315"/>
-      <c r="J15" s="311"/>
-      <c r="K15" s="295"/>
+      <c r="I15" s="316"/>
+      <c r="J15" s="312"/>
+      <c r="K15" s="294"/>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="123" t="s">
@@ -8765,13 +8763,13 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="320" t="s">
+      <c r="A21" s="321" t="s">
         <v>258</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -8786,11 +8784,11 @@
       <c r="Q21" s="10"/>
     </row>
     <row r="22" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -9039,10 +9037,10 @@
         <f>ROUND((B32-31000)*0.42+5950,2)</f>
         <v>10076.74</v>
       </c>
-      <c r="C33" s="298" t="s">
+      <c r="C33" s="299" t="s">
         <v>205</v>
       </c>
-      <c r="D33" s="295"/>
+      <c r="D33" s="294"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -9065,10 +9063,10 @@
         <f>ROUND((B13+H13-620)*0.06,2)</f>
         <v>337.3</v>
       </c>
-      <c r="C34" s="298" t="s">
+      <c r="C34" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="295"/>
+      <c r="D34" s="294"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -9365,10 +9363,10 @@
       <c r="Q47" s="10"/>
     </row>
     <row r="48" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="301" t="s">
+      <c r="A48" s="302" t="s">
         <v>262</v>
       </c>
-      <c r="B48" s="291"/>
+      <c r="B48" s="290"/>
       <c r="C48" s="10"/>
       <c r="D48" s="10"/>
       <c r="E48" s="10"/>
@@ -11337,62 +11335,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="317" t="s">
+      <c r="A1" s="318" t="s">
         <v>272</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="318" t="s">
+      <c r="G1" s="319" t="s">
         <v>273</v>
       </c>
-      <c r="H1" s="303"/>
-      <c r="I1" s="303"/>
-      <c r="J1" s="303"/>
-      <c r="K1" s="291"/>
+      <c r="H1" s="304"/>
+      <c r="I1" s="304"/>
+      <c r="J1" s="304"/>
+      <c r="K1" s="290"/>
       <c r="L1" s="118"/>
-      <c r="M1" s="318" t="s">
+      <c r="M1" s="319" t="s">
         <v>274</v>
       </c>
-      <c r="N1" s="303"/>
-      <c r="O1" s="303"/>
-      <c r="P1" s="303"/>
-      <c r="Q1" s="291"/>
+      <c r="N1" s="304"/>
+      <c r="O1" s="304"/>
+      <c r="P1" s="304"/>
+      <c r="Q1" s="290"/>
       <c r="R1" s="118"/>
-      <c r="S1" s="318" t="s">
+      <c r="S1" s="319" t="s">
         <v>275</v>
       </c>
-      <c r="T1" s="303"/>
-      <c r="U1" s="303"/>
-      <c r="V1" s="303"/>
-      <c r="W1" s="291"/>
+      <c r="T1" s="304"/>
+      <c r="U1" s="304"/>
+      <c r="V1" s="304"/>
+      <c r="W1" s="290"/>
     </row>
     <row r="2" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="297"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="298"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="297"/>
-      <c r="H2" s="297"/>
-      <c r="I2" s="297"/>
-      <c r="J2" s="297"/>
-      <c r="K2" s="300"/>
+      <c r="G2" s="298"/>
+      <c r="H2" s="298"/>
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="301"/>
       <c r="L2" s="118"/>
-      <c r="M2" s="297"/>
-      <c r="N2" s="297"/>
-      <c r="O2" s="297"/>
-      <c r="P2" s="297"/>
-      <c r="Q2" s="300"/>
+      <c r="M2" s="298"/>
+      <c r="N2" s="298"/>
+      <c r="O2" s="298"/>
+      <c r="P2" s="298"/>
+      <c r="Q2" s="301"/>
       <c r="R2" s="118"/>
-      <c r="S2" s="297"/>
-      <c r="T2" s="297"/>
-      <c r="U2" s="297"/>
-      <c r="V2" s="297"/>
-      <c r="W2" s="300"/>
+      <c r="S2" s="298"/>
+      <c r="T2" s="298"/>
+      <c r="U2" s="298"/>
+      <c r="V2" s="298"/>
+      <c r="W2" s="301"/>
     </row>
     <row r="3" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -11913,9 +11911,9 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="315"/>
-      <c r="J15" s="311"/>
-      <c r="K15" s="295"/>
+      <c r="I15" s="316"/>
+      <c r="J15" s="312"/>
+      <c r="K15" s="294"/>
       <c r="L15" s="10"/>
       <c r="M15" s="240" t="s">
         <v>11</v>
@@ -12095,13 +12093,13 @@
       <c r="W20" s="10"/>
     </row>
     <row r="21" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="320" t="s">
+      <c r="A21" s="321" t="s">
         <v>280</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -12121,11 +12119,11 @@
       <c r="W21" s="10"/>
     </row>
     <row r="22" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -12325,10 +12323,10 @@
         <f>ROUND((B30-60000)*0.48+1400+4225+12180,2)</f>
         <v>27569.02</v>
       </c>
-      <c r="C31" s="321" t="s">
+      <c r="C31" s="322" t="s">
         <v>282</v>
       </c>
-      <c r="D31" s="295"/>
+      <c r="D31" s="294"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
@@ -12351,10 +12349,10 @@
         <f>ROUND((B13+H13+N13-620)*0.06,2)</f>
         <v>420.11</v>
       </c>
-      <c r="C32" s="298" t="s">
+      <c r="C32" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="295"/>
+      <c r="D32" s="294"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
@@ -12580,12 +12578,12 @@
         <v>284</v>
       </c>
       <c r="D42" s="10"/>
-      <c r="E42" s="322" t="s">
+      <c r="E42" s="323" t="s">
         <v>285</v>
       </c>
-      <c r="F42" s="311"/>
-      <c r="G42" s="311"/>
-      <c r="H42" s="295"/>
+      <c r="F42" s="312"/>
+      <c r="G42" s="312"/>
+      <c r="H42" s="294"/>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
       <c r="K42" s="10"/>
@@ -12676,10 +12674,10 @@
       <c r="Q45" s="10"/>
     </row>
     <row r="46" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="301" t="s">
+      <c r="A46" s="302" t="s">
         <v>289</v>
       </c>
-      <c r="B46" s="291"/>
+      <c r="B46" s="290"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="248" t="s">
@@ -13952,21 +13950,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="317" t="s">
+      <c r="A1" s="318" t="s">
         <v>297</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
     </row>
     <row r="2" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="297"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="298"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
     </row>
     <row r="3" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14182,21 +14180,21 @@
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="320" t="s">
+      <c r="A21" s="321" t="s">
         <v>298</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
     </row>
     <row r="22" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
     </row>
     <row r="23" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -14297,10 +14295,10 @@
         <f>ROUND((B30-93120)*0.5+32571.75,2)</f>
         <v>34026.410000000003</v>
       </c>
-      <c r="C31" s="321" t="s">
+      <c r="C31" s="322" t="s">
         <v>23</v>
       </c>
-      <c r="D31" s="295"/>
+      <c r="D31" s="294"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
     </row>
@@ -14312,10 +14310,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>894.01</v>
       </c>
-      <c r="C32" s="298" t="s">
+      <c r="C32" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="295"/>
+      <c r="D32" s="294"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
     </row>
@@ -14427,22 +14425,22 @@
         <f>B39-B40</f>
         <v>-924.99999999999625</v>
       </c>
-      <c r="C42" s="292" t="s">
+      <c r="C42" s="291" t="s">
         <v>300</v>
       </c>
-      <c r="D42" s="295"/>
-      <c r="E42" s="323" t="s">
+      <c r="D42" s="294"/>
+      <c r="E42" s="324" t="s">
         <v>33</v>
       </c>
-      <c r="F42" s="311"/>
+      <c r="F42" s="312"/>
     </row>
     <row r="43" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="57"/>
       <c r="B43" s="57"/>
-      <c r="C43" s="324" t="s">
+      <c r="C43" s="325" t="s">
         <v>301</v>
       </c>
-      <c r="D43" s="295"/>
+      <c r="D43" s="294"/>
       <c r="E43" s="248" t="s">
         <v>34</v>
       </c>
@@ -14478,10 +14476,10 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="301" t="s">
+      <c r="A46" s="302" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="291"/>
+      <c r="B46" s="290"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="248" t="s">
@@ -15732,21 +15730,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="317" t="s">
+      <c r="A1" s="318" t="s">
         <v>311</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
     </row>
     <row r="2" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="297"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="298"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
     </row>
     <row r="3" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -15962,21 +15960,21 @@
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="320" t="s">
+      <c r="A21" s="321" t="s">
         <v>312</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
     </row>
     <row r="22" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
     </row>
     <row r="23" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -16117,10 +16115,10 @@
         <f>ROUND((B33-99266)*0.5+34222.42,2)</f>
         <v>44541.03</v>
       </c>
-      <c r="C34" s="321" t="s">
+      <c r="C34" s="322" t="s">
         <v>23</v>
       </c>
-      <c r="D34" s="295"/>
+      <c r="D34" s="294"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
     </row>
@@ -16132,10 +16130,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>1186.67</v>
       </c>
-      <c r="C35" s="298" t="s">
+      <c r="C35" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="295"/>
+      <c r="D35" s="294"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
     </row>
@@ -16247,14 +16245,14 @@
         <f>B42-B43</f>
         <v>-646.00000000000227</v>
       </c>
-      <c r="C45" s="292" t="s">
+      <c r="C45" s="291" t="s">
         <v>315</v>
       </c>
-      <c r="D45" s="295"/>
-      <c r="E45" s="323" t="s">
+      <c r="D45" s="294"/>
+      <c r="E45" s="324" t="s">
         <v>33</v>
       </c>
-      <c r="F45" s="311"/>
+      <c r="F45" s="312"/>
     </row>
     <row r="46" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="57"/>
@@ -16298,10 +16296,10 @@
       </c>
     </row>
     <row r="49" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="301" t="s">
+      <c r="A49" s="302" t="s">
         <v>37</v>
       </c>
-      <c r="B49" s="291"/>
+      <c r="B49" s="290"/>
       <c r="C49" s="10"/>
       <c r="D49" s="10"/>
       <c r="E49" s="248" t="s">
@@ -18536,7 +18534,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.25" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53.25" customWidth="1"/>
@@ -18833,10 +18831,10 @@
         <f>ROUND((B29-103072)*0.5+35534.38,2)</f>
         <v>52245.8</v>
       </c>
-      <c r="C30" s="292" t="s">
+      <c r="C30" s="291" t="s">
         <v>23</v>
       </c>
-      <c r="D30" s="293"/>
+      <c r="D30" s="292"/>
     </row>
     <row r="31" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="52" t="s">
@@ -18846,10 +18844,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>1301.33</v>
       </c>
-      <c r="C31" s="294" t="s">
+      <c r="C31" s="293" t="s">
         <v>25</v>
       </c>
-      <c r="D31" s="293"/>
+      <c r="D31" s="292"/>
     </row>
     <row r="32" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="82" t="s">
@@ -18931,10 +18929,10 @@
         <f>B38</f>
         <v>-649.99999999999773</v>
       </c>
-      <c r="C40" s="292" t="s">
+      <c r="C40" s="291" t="s">
         <v>32</v>
       </c>
-      <c r="D40" s="295"/>
+      <c r="D40" s="294"/>
     </row>
     <row r="41" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="57"/>
@@ -18944,256 +18942,251 @@
       </c>
       <c r="D41" s="60"/>
     </row>
-    <row r="42" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="290" t="s">
+    <row r="42" spans="1:4" s="346" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="289" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="291"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
+      <c r="B42" s="289"/>
+      <c r="C42" s="289"/>
+      <c r="D42" s="60"/>
     </row>
     <row r="43" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="88" t="s">
+      <c r="A43" s="289"/>
+      <c r="B43" s="289"/>
+      <c r="C43" s="289"/>
+      <c r="D43" s="10"/>
+    </row>
+    <row r="44" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="88" t="s">
         <v>40</v>
       </c>
-      <c r="B43" s="62">
+      <c r="B44" s="62">
         <f>B4</f>
         <v>177796.22</v>
       </c>
-      <c r="C43" s="60"/>
-      <c r="D43" s="10"/>
-    </row>
-    <row r="44" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="90" t="s">
+      <c r="C44" s="60"/>
+      <c r="D44" s="10"/>
+    </row>
+    <row r="45" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="129">
+      <c r="B45" s="129">
         <f>B10</f>
         <v>16213.27</v>
       </c>
-      <c r="C44" s="60"/>
-      <c r="D44" s="119"/>
-    </row>
-    <row r="45" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="90" t="s">
+      <c r="C45" s="60"/>
+      <c r="D45" s="119"/>
+    </row>
+    <row r="46" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B45" s="129">
+      <c r="B46" s="129">
         <f>B34</f>
         <v>53044.130000000005</v>
       </c>
-      <c r="C45" s="60"/>
-      <c r="D45" s="119"/>
-    </row>
-    <row r="46" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="88" t="s">
+      <c r="C46" s="60"/>
+      <c r="D46" s="119"/>
+    </row>
+    <row r="47" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="88" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="62">
+      <c r="B47" s="62">
         <f>0-'2025'!B12</f>
         <v>-42.48</v>
       </c>
-      <c r="C46" s="60"/>
-      <c r="D46" s="119"/>
-    </row>
-    <row r="47" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="92" t="s">
-        <v>51</v>
-      </c>
-      <c r="B47" s="84"/>
       <c r="C47" s="60"/>
       <c r="D47" s="119"/>
     </row>
-    <row r="48" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="283" t="s">
+    <row r="48" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="92" t="s">
+        <v>51</v>
+      </c>
+      <c r="B48" s="84"/>
+      <c r="C48" s="60"/>
+      <c r="D48" s="119"/>
+    </row>
+    <row r="49" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="283" t="s">
         <v>54</v>
       </c>
-      <c r="B48" s="282">
-        <f>B43-B44-B45+B46</f>
+      <c r="B49" s="282">
+        <f>B44-B45-B46+B47</f>
         <v>108496.34000000001</v>
       </c>
-      <c r="C48" s="72"/>
-      <c r="D48" s="119"/>
-    </row>
-    <row r="50" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="345" t="s">
+      <c r="C49" s="72"/>
+      <c r="D49" s="119"/>
+    </row>
+    <row r="51" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="295" t="s">
         <v>458</v>
       </c>
-      <c r="B50" s="346"/>
-      <c r="C50" s="346"/>
-      <c r="D50" s="346"/>
-    </row>
-    <row r="51" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="248" t="s">
-        <v>457</v>
-      </c>
-      <c r="B51" s="235">
-        <f>(SUM(B64:B66)+SUM(C64:C68))*0.89</f>
-        <v>66640.031599999988</v>
-      </c>
+      <c r="B51" s="296"/>
+      <c r="C51" s="296"/>
+      <c r="D51" s="296"/>
     </row>
     <row r="52" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="248" t="s">
+        <v>457</v>
+      </c>
+      <c r="B52" s="235">
+        <f>(SUM(B65:B67)+SUM(C65:C69))*0.89</f>
+        <v>66640.031599999988</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="248" t="s">
         <v>460</v>
       </c>
-      <c r="B52" s="253">
-        <f>SUM(B56:B61)+SUM(D56:D61)</f>
+      <c r="B53" s="253">
+        <f>SUM(B57:B62)+SUM(D57:D62)</f>
         <v>110952.88999999998</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="266" t="s">
+    <row r="54" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="266" t="s">
         <v>36</v>
       </c>
-      <c r="B53" s="267">
-        <f>B51+B52</f>
+      <c r="B54" s="267">
+        <f>B52+B53</f>
         <v>177592.92159999997</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="285" t="s">
+    <row r="56" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="285" t="s">
         <v>459</v>
       </c>
-      <c r="B55" s="286"/>
-      <c r="C55" s="286"/>
-      <c r="D55" s="286"/>
-    </row>
-    <row r="56" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="280" t="s">
-        <v>38</v>
-      </c>
-      <c r="B56" s="279">
-        <v>6773</v>
-      </c>
-      <c r="C56" s="275" t="s">
-        <v>39</v>
-      </c>
-      <c r="D56" s="279">
-        <v>7518.44</v>
-      </c>
+      <c r="B56" s="286"/>
+      <c r="C56" s="286"/>
+      <c r="D56" s="286"/>
     </row>
     <row r="57" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="280" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B57" s="279">
-        <v>7341.69</v>
+        <v>6773</v>
       </c>
       <c r="C57" s="275" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D57" s="279">
-        <v>6637.88</v>
+        <v>7518.44</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="280" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B58" s="279">
-        <v>7121.67</v>
+        <v>7341.69</v>
       </c>
       <c r="C58" s="275" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D58" s="279">
-        <v>6888.36</v>
+        <v>6637.88</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="280" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B59" s="279">
-        <v>7138.6</v>
+        <v>7121.67</v>
       </c>
       <c r="C59" s="275" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D59" s="279">
-        <v>17811.8</v>
+        <v>6888.36</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="280" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B60" s="279">
-        <v>6773.36</v>
+        <v>7138.6</v>
       </c>
       <c r="C60" s="275" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D60" s="279">
-        <v>15441.21</v>
+        <v>17811.8</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="280" t="s">
+        <v>49</v>
+      </c>
+      <c r="B61" s="279">
+        <v>6773.36</v>
+      </c>
+      <c r="C61" s="275" t="s">
+        <v>50</v>
+      </c>
+      <c r="D61" s="279">
+        <v>15441.21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="280" t="s">
         <v>52</v>
       </c>
-      <c r="B61" s="279">
+      <c r="B62" s="279">
         <v>13789.38</v>
       </c>
-      <c r="C61" s="275" t="s">
+      <c r="C62" s="275" t="s">
         <v>53</v>
       </c>
-      <c r="D61" s="279">
+      <c r="D62" s="279">
         <v>7717.5</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="249"/>
-    </row>
     <row r="63" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="287" t="s">
+      <c r="A63" s="249"/>
+    </row>
+    <row r="64" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="287" t="s">
         <v>452</v>
       </c>
-      <c r="B63" s="288"/>
-      <c r="C63" s="288"/>
-    </row>
-    <row r="64" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="281" t="s">
-        <v>453</v>
-      </c>
-      <c r="B64" s="276">
-        <v>19337.919999999998</v>
-      </c>
-      <c r="C64" s="276">
-        <v>27198.92</v>
-      </c>
+      <c r="B64" s="288"/>
+      <c r="C64" s="288"/>
     </row>
     <row r="65" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="281" t="s">
-        <v>454</v>
-      </c>
-      <c r="B65" s="277">
-        <v>5294.12</v>
-      </c>
-      <c r="C65" s="278">
-        <v>6534.84</v>
+        <v>453</v>
+      </c>
+      <c r="B65" s="276">
+        <v>19337.919999999998</v>
+      </c>
+      <c r="C65" s="276">
+        <v>27198.92</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="281" t="s">
-        <v>455</v>
-      </c>
-      <c r="B66" s="278">
-        <v>7497.68</v>
+        <v>454</v>
+      </c>
+      <c r="B66" s="277">
+        <v>5294.12</v>
       </c>
       <c r="C66" s="278">
-        <v>9012.9599999999991</v>
+        <v>6534.84</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="281" t="s">
-        <v>456</v>
-      </c>
-      <c r="B67" s="276">
-        <v>0</v>
-      </c>
-      <c r="C67" s="276">
-        <v>0</v>
+        <v>455</v>
+      </c>
+      <c r="B67" s="278">
+        <v>7497.68</v>
+      </c>
+      <c r="C67" s="278">
+        <v>9012.9599999999991</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -19207,17 +19200,28 @@
         <v>0</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="281" t="s">
+        <v>456</v>
+      </c>
+      <c r="B69" s="276">
+        <v>0</v>
+      </c>
+      <c r="C69" s="276">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A63:C63"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A64:C64"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A18:C19"/>
-    <mergeCell ref="A42:B42"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="C40:D40"/>
-    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A42:C43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19688,11 +19692,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="338" t="s">
+      <c r="A1" s="334" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="339"/>
-      <c r="C1" s="340"/>
+      <c r="B1" s="335"/>
+      <c r="C1" s="336"/>
       <c r="D1" s="159"/>
       <c r="E1" s="39" t="s">
         <v>327</v>
@@ -19860,11 +19864,11 @@
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="335" t="s">
+      <c r="A11" s="327" t="s">
         <v>343</v>
       </c>
-      <c r="B11" s="336"/>
-      <c r="C11" s="337"/>
+      <c r="B11" s="328"/>
+      <c r="C11" s="329"/>
       <c r="D11" s="159"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -20048,11 +20052,11 @@
       <c r="J22" s="10"/>
     </row>
     <row r="23" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="335" t="s">
+      <c r="A23" s="327" t="s">
         <v>354</v>
       </c>
-      <c r="B23" s="336"/>
-      <c r="C23" s="337"/>
+      <c r="B23" s="328"/>
+      <c r="C23" s="329"/>
       <c r="D23" s="159"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -20328,11 +20332,11 @@
       <c r="J39" s="10"/>
     </row>
     <row r="40" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="342" t="s">
+      <c r="A40" s="338" t="s">
         <v>370</v>
       </c>
-      <c r="B40" s="343"/>
-      <c r="C40" s="344"/>
+      <c r="B40" s="339"/>
+      <c r="C40" s="340"/>
       <c r="D40" s="159"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -20424,13 +20428,13 @@
       <c r="C46" s="212">
         <v>-604</v>
       </c>
-      <c r="D46" s="334"/>
-      <c r="E46" s="311"/>
-      <c r="F46" s="311"/>
-      <c r="G46" s="311"/>
-      <c r="H46" s="311"/>
-      <c r="I46" s="311"/>
-      <c r="J46" s="295"/>
+      <c r="D46" s="326"/>
+      <c r="E46" s="312"/>
+      <c r="F46" s="312"/>
+      <c r="G46" s="312"/>
+      <c r="H46" s="312"/>
+      <c r="I46" s="312"/>
+      <c r="J46" s="294"/>
     </row>
     <row r="47" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="175" t="s">
@@ -20564,11 +20568,11 @@
       <c r="J54" s="10"/>
     </row>
     <row r="55" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="329" t="s">
+      <c r="A55" s="341" t="s">
         <v>382</v>
       </c>
-      <c r="B55" s="330"/>
-      <c r="C55" s="331"/>
+      <c r="B55" s="342"/>
+      <c r="C55" s="343"/>
       <c r="D55" s="215"/>
       <c r="E55" s="10"/>
       <c r="F55" s="10"/>
@@ -20879,10 +20883,10 @@
       <c r="J75" s="10"/>
     </row>
     <row r="76" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="341" t="s">
+      <c r="A76" s="337" t="s">
         <v>398</v>
       </c>
-      <c r="B76" s="297"/>
+      <c r="B76" s="298"/>
       <c r="C76" s="60"/>
       <c r="D76" s="10"/>
       <c r="E76" s="10"/>
@@ -20893,8 +20897,8 @@
       <c r="J76" s="10"/>
     </row>
     <row r="77" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="314"/>
-      <c r="B77" s="297"/>
+      <c r="A77" s="315"/>
+      <c r="B77" s="298"/>
       <c r="C77" s="60"/>
       <c r="D77" s="10"/>
       <c r="E77" s="10"/>
@@ -20933,10 +20937,10 @@
       <c r="J79" s="10"/>
     </row>
     <row r="80" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="332" t="s">
+      <c r="A80" s="344" t="s">
         <v>401</v>
       </c>
-      <c r="B80" s="305"/>
+      <c r="B80" s="306"/>
       <c r="C80" s="60"/>
       <c r="D80" s="10"/>
       <c r="E80" s="10"/>
@@ -20947,8 +20951,8 @@
       <c r="J80" s="10"/>
     </row>
     <row r="81" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="314"/>
-      <c r="B81" s="297"/>
+      <c r="A81" s="315"/>
+      <c r="B81" s="298"/>
       <c r="C81" s="60"/>
       <c r="D81" s="10"/>
       <c r="E81" s="10"/>
@@ -21155,10 +21159,10 @@
       <c r="J95" s="10"/>
     </row>
     <row r="96" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="325" t="s">
+      <c r="A96" s="330" t="s">
         <v>416</v>
       </c>
-      <c r="B96" s="326"/>
+      <c r="B96" s="331"/>
       <c r="C96" s="10"/>
       <c r="D96" s="10"/>
       <c r="E96" s="10"/>
@@ -21169,8 +21173,8 @@
       <c r="J96" s="10"/>
     </row>
     <row r="97" spans="1:10" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="327"/>
-      <c r="B97" s="328"/>
+      <c r="A97" s="332"/>
+      <c r="B97" s="333"/>
       <c r="C97" s="10"/>
       <c r="D97" s="10"/>
       <c r="E97" s="10"/>
@@ -21319,14 +21323,14 @@
       <c r="B108" s="10"/>
     </row>
     <row r="109" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="333" t="s">
+      <c r="A109" s="345" t="s">
         <v>428</v>
       </c>
-      <c r="B109" s="326"/>
+      <c r="B109" s="331"/>
     </row>
     <row r="110" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="327"/>
-      <c r="B110" s="328"/>
+      <c r="A110" s="332"/>
+      <c r="B110" s="333"/>
     </row>
     <row r="111" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="236" t="s">
@@ -21398,14 +21402,14 @@
       </c>
     </row>
     <row r="124" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="325" t="s">
+      <c r="A124" s="330" t="s">
         <v>442</v>
       </c>
-      <c r="B124" s="326"/>
+      <c r="B124" s="331"/>
     </row>
     <row r="125" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="327"/>
-      <c r="B125" s="328"/>
+      <c r="A125" s="332"/>
+      <c r="B125" s="333"/>
     </row>
     <row r="126" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="225" t="s">
@@ -21424,14 +21428,14 @@
       </c>
     </row>
     <row r="128" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="325" t="s">
+      <c r="A128" s="330" t="s">
         <v>447</v>
       </c>
-      <c r="B128" s="326"/>
+      <c r="B128" s="331"/>
     </row>
     <row r="129" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="327"/>
-      <c r="B129" s="328"/>
+      <c r="A129" s="332"/>
+      <c r="B129" s="333"/>
     </row>
     <row r="130" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="225" t="s">
@@ -21451,6 +21455,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A124:B125"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A80:B81"/>
+    <mergeCell ref="A128:B129"/>
+    <mergeCell ref="A109:B110"/>
     <mergeCell ref="D46:J46"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A96:B97"/>
@@ -21458,11 +21467,6 @@
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A76:B77"/>
     <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A124:B125"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A80:B81"/>
-    <mergeCell ref="A128:B129"/>
-    <mergeCell ref="A109:B110"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
@@ -22623,20 +22627,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="302" t="s">
+      <c r="A1" s="303" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="291"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="290"/>
     </row>
     <row r="2" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="299"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="300"/>
+      <c r="A2" s="300"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="301"/>
     </row>
     <row r="3" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -22796,11 +22800,11 @@
       <c r="B15" s="59">
         <v>438.04</v>
       </c>
-      <c r="C15" s="310" t="s">
+      <c r="C15" s="311" t="s">
         <v>132</v>
       </c>
-      <c r="D15" s="311"/>
-      <c r="E15" s="295"/>
+      <c r="D15" s="312"/>
+      <c r="E15" s="294"/>
     </row>
     <row r="16" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="58" t="s">
@@ -22848,20 +22852,20 @@
       <c r="E20" s="49"/>
     </row>
     <row r="21" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="304" t="s">
+      <c r="A21" s="305" t="s">
         <v>134</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
     </row>
     <row r="22" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
     </row>
     <row r="23" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="63" t="s">
@@ -22989,10 +22993,10 @@
         <f>ROUND((B33-18000)*0.35+1750,2)</f>
         <v>5779.41</v>
       </c>
-      <c r="C34" s="298" t="s">
+      <c r="C34" s="299" t="s">
         <v>141</v>
       </c>
-      <c r="D34" s="295"/>
+      <c r="D34" s="294"/>
       <c r="E34" s="10"/>
     </row>
     <row r="35" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -23003,10 +23007,10 @@
         <f>ROUND((B13-620)*0.06,2)</f>
         <v>244.34</v>
       </c>
-      <c r="C35" s="298" t="s">
+      <c r="C35" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="295"/>
+      <c r="D35" s="294"/>
       <c r="E35" s="10"/>
     </row>
     <row r="36" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -23133,10 +23137,10 @@
       <c r="E48" s="10"/>
     </row>
     <row r="49" spans="1:5" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="301" t="s">
+      <c r="A49" s="302" t="s">
         <v>146</v>
       </c>
-      <c r="B49" s="291"/>
+      <c r="B49" s="290"/>
       <c r="C49" s="10"/>
       <c r="D49" s="10"/>
       <c r="E49" s="10"/>
@@ -26507,34 +26511,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="313" t="s">
+      <c r="A1" s="314" t="s">
         <v>197</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="312" t="s">
+      <c r="G1" s="313" t="s">
         <v>198</v>
       </c>
-      <c r="H1" s="303"/>
-      <c r="I1" s="303"/>
-      <c r="J1" s="303"/>
-      <c r="K1" s="291"/>
+      <c r="H1" s="304"/>
+      <c r="I1" s="304"/>
+      <c r="J1" s="304"/>
+      <c r="K1" s="290"/>
     </row>
     <row r="2" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="314"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="315"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="297"/>
-      <c r="H2" s="297"/>
-      <c r="I2" s="297"/>
-      <c r="J2" s="297"/>
-      <c r="K2" s="300"/>
+      <c r="G2" s="298"/>
+      <c r="H2" s="298"/>
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="301"/>
     </row>
     <row r="3" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -26833,11 +26837,11 @@
       <c r="B15" s="59">
         <v>1535.69</v>
       </c>
-      <c r="C15" s="310" t="s">
+      <c r="C15" s="311" t="s">
         <v>132</v>
       </c>
-      <c r="D15" s="311"/>
-      <c r="E15" s="295"/>
+      <c r="D15" s="312"/>
+      <c r="E15" s="294"/>
       <c r="F15" s="119"/>
       <c r="G15" s="123" t="s">
         <v>131</v>
@@ -26845,11 +26849,11 @@
       <c r="H15" s="59">
         <v>413.13</v>
       </c>
-      <c r="I15" s="310" t="s">
+      <c r="I15" s="311" t="s">
         <v>132</v>
       </c>
-      <c r="J15" s="311"/>
-      <c r="K15" s="295"/>
+      <c r="J15" s="312"/>
+      <c r="K15" s="294"/>
     </row>
     <row r="16" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="58" t="s">
@@ -26937,13 +26941,13 @@
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="304" t="s">
+      <c r="A21" s="305" t="s">
         <v>202</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -26952,11 +26956,11 @@
       <c r="K21" s="10"/>
     </row>
     <row r="22" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -27157,10 +27161,10 @@
         <f>ROUND((B33-31000)*0.42+6300,2)</f>
         <v>7196.73</v>
       </c>
-      <c r="C34" s="298" t="s">
+      <c r="C34" s="299" t="s">
         <v>205</v>
       </c>
-      <c r="D34" s="295"/>
+      <c r="D34" s="294"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -27177,10 +27181,10 @@
         <f>ROUND((B13+H13-620)*0.06,2)</f>
         <v>312.08999999999997</v>
       </c>
-      <c r="C35" s="298" t="s">
+      <c r="C35" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="295"/>
+      <c r="D35" s="294"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
@@ -27404,10 +27408,10 @@
       <c r="K49" s="10"/>
     </row>
     <row r="50" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="301" t="s">
+      <c r="A50" s="302" t="s">
         <v>207</v>
       </c>
-      <c r="B50" s="291"/>
+      <c r="B50" s="290"/>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
@@ -31169,48 +31173,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="313" t="s">
+      <c r="A1" s="314" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="303"/>
-      <c r="C1" s="303"/>
-      <c r="D1" s="303"/>
-      <c r="E1" s="303"/>
+      <c r="B1" s="304"/>
+      <c r="C1" s="304"/>
+      <c r="D1" s="304"/>
+      <c r="E1" s="304"/>
       <c r="F1" s="118"/>
-      <c r="G1" s="316" t="s">
+      <c r="G1" s="317" t="s">
         <v>221</v>
       </c>
-      <c r="H1" s="303"/>
-      <c r="I1" s="303"/>
-      <c r="J1" s="303"/>
-      <c r="K1" s="303"/>
+      <c r="H1" s="304"/>
+      <c r="I1" s="304"/>
+      <c r="J1" s="304"/>
+      <c r="K1" s="304"/>
       <c r="L1" s="118"/>
-      <c r="M1" s="312" t="s">
+      <c r="M1" s="313" t="s">
         <v>222</v>
       </c>
-      <c r="N1" s="303"/>
-      <c r="O1" s="303"/>
-      <c r="P1" s="303"/>
-      <c r="Q1" s="291"/>
+      <c r="N1" s="304"/>
+      <c r="O1" s="304"/>
+      <c r="P1" s="304"/>
+      <c r="Q1" s="290"/>
     </row>
     <row r="2" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="314"/>
-      <c r="B2" s="297"/>
-      <c r="C2" s="297"/>
-      <c r="D2" s="297"/>
-      <c r="E2" s="297"/>
+      <c r="A2" s="315"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="118"/>
-      <c r="G2" s="297"/>
-      <c r="H2" s="297"/>
-      <c r="I2" s="297"/>
-      <c r="J2" s="297"/>
-      <c r="K2" s="297"/>
+      <c r="G2" s="298"/>
+      <c r="H2" s="298"/>
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="298"/>
       <c r="L2" s="118"/>
-      <c r="M2" s="297"/>
-      <c r="N2" s="297"/>
-      <c r="O2" s="297"/>
-      <c r="P2" s="297"/>
-      <c r="Q2" s="300"/>
+      <c r="M2" s="298"/>
+      <c r="N2" s="298"/>
+      <c r="O2" s="298"/>
+      <c r="P2" s="298"/>
+      <c r="Q2" s="301"/>
     </row>
     <row r="3" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37"/>
@@ -31648,11 +31652,11 @@
       <c r="B15" s="59">
         <v>175.89</v>
       </c>
-      <c r="C15" s="310" t="s">
+      <c r="C15" s="311" t="s">
         <v>132</v>
       </c>
-      <c r="D15" s="311"/>
-      <c r="E15" s="295"/>
+      <c r="D15" s="312"/>
+      <c r="E15" s="294"/>
       <c r="F15" s="119"/>
       <c r="G15" s="123" t="s">
         <v>131</v>
@@ -31660,17 +31664,17 @@
       <c r="H15" s="59">
         <v>13.93</v>
       </c>
-      <c r="I15" s="310" t="s">
+      <c r="I15" s="311" t="s">
         <v>132</v>
       </c>
-      <c r="J15" s="311"/>
-      <c r="K15" s="295"/>
+      <c r="J15" s="312"/>
+      <c r="K15" s="294"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="O15" s="315"/>
-      <c r="P15" s="311"/>
-      <c r="Q15" s="295"/>
+      <c r="O15" s="316"/>
+      <c r="P15" s="312"/>
+      <c r="Q15" s="294"/>
     </row>
     <row r="16" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="58" t="s">
@@ -31794,13 +31798,13 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="304" t="s">
+      <c r="A21" s="305" t="s">
         <v>226</v>
       </c>
-      <c r="B21" s="305"/>
-      <c r="C21" s="305"/>
-      <c r="D21" s="305"/>
-      <c r="E21" s="306"/>
+      <c r="B21" s="306"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="307"/>
       <c r="F21" s="72"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -31815,11 +31819,11 @@
       <c r="Q21" s="10"/>
     </row>
     <row r="22" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="307"/>
-      <c r="B22" s="308"/>
-      <c r="C22" s="308"/>
-      <c r="D22" s="308"/>
-      <c r="E22" s="309"/>
+      <c r="A22" s="308"/>
+      <c r="B22" s="309"/>
+      <c r="C22" s="309"/>
+      <c r="D22" s="309"/>
+      <c r="E22" s="310"/>
       <c r="F22" s="72"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -32068,10 +32072,10 @@
         <f>ROUND((B32-31000)*0.42+6300,2)</f>
         <v>8538.18</v>
       </c>
-      <c r="C33" s="298" t="s">
+      <c r="C33" s="299" t="s">
         <v>205</v>
       </c>
-      <c r="D33" s="295"/>
+      <c r="D33" s="294"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -32094,10 +32098,10 @@
         <f>ROUND((B13+H13+N13-620)*0.06,2)</f>
         <v>329.36</v>
       </c>
-      <c r="C34" s="298" t="s">
+      <c r="C34" s="299" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="295"/>
+      <c r="D34" s="294"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -32375,10 +32379,10 @@
       <c r="Q46" s="10"/>
     </row>
     <row r="47" spans="1:17" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="301" t="s">
+      <c r="A47" s="302" t="s">
         <v>229</v>
       </c>
-      <c r="B47" s="291"/>
+      <c r="B47" s="290"/>
       <c r="C47" s="10"/>
       <c r="D47" s="10"/>
       <c r="E47" s="10"/>

</xml_diff>